<commit_message>
Add pull-ozon-stock command; set initial stock for new drafts
- ozon_client.get_stocks() / catalog_editor.stock_from_ozon_item() +
  fill_empty_stock(): one-off pull of live Ozon stock (FBO+FBS present)
  into "Кол-во к продаже" for existing products where it's still empty —
  never overwrites cells already set locally. New --pull-ozon-stock
  command (main.py + main.yml); response field names aren't verified on
  live data yet, so the command prints the raw response for the first
  items on first real run for a sanity check.
- ozon_new_products.xlsx: set quantity_to_sell = 50 for all new drafts,
  except the DQ250 mechatronic-with-board (02E927770AL) = 3, per request.
</commit_message>
<xml_diff>
--- a/data/master_control.xlsx
+++ b/data/master_control.xlsx
@@ -3302,7 +3302,9 @@
       <c r="I5" s="2" t="n">
         <v>145000</v>
       </c>
-      <c r="J5" s="2" t="n"/>
+      <c r="J5" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
@@ -5771,7 +5773,9 @@
       <c r="I52" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J52" s="2" t="n"/>
+      <c r="J52" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="inlineStr">
         <is>
@@ -5873,7 +5877,9 @@
       <c r="I54" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J54" s="2" t="n"/>
+      <c r="J54" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
@@ -6700,7 +6706,9 @@
       <c r="I70" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J70" s="2" t="n"/>
+      <c r="J70" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K70" s="2" t="n"/>
       <c r="L70" s="2" t="inlineStr">
         <is>
@@ -7309,7 +7317,9 @@
       <c r="I83" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J83" s="2" t="n"/>
+      <c r="J83" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K83" s="2" t="n"/>
       <c r="L83" s="2" t="inlineStr">
         <is>
@@ -7360,7 +7370,9 @@
       <c r="I84" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J84" s="2" t="n"/>
+      <c r="J84" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K84" s="2" t="n"/>
       <c r="L84" s="2" t="inlineStr">
         <is>
@@ -7462,7 +7474,9 @@
       <c r="I86" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J86" s="2" t="n"/>
+      <c r="J86" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K86" s="2" t="n"/>
       <c r="L86" s="2" t="inlineStr">
         <is>
@@ -7513,7 +7527,9 @@
       <c r="I87" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J87" s="2" t="n"/>
+      <c r="J87" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K87" s="2" t="n"/>
       <c r="L87" s="2" t="inlineStr">
         <is>
@@ -7611,7 +7627,9 @@
       <c r="I89" s="2" t="n">
         <v>4000</v>
       </c>
-      <c r="J89" s="2" t="n"/>
+      <c r="J89" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K89" s="2" t="n"/>
       <c r="L89" s="2" t="inlineStr">
         <is>
@@ -7662,7 +7680,9 @@
       <c r="I90" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="J90" s="2" t="n"/>
+      <c r="J90" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K90" s="2" t="n"/>
       <c r="L90" s="2" t="inlineStr">
         <is>
@@ -7713,7 +7733,9 @@
       <c r="I91" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J91" s="2" t="n"/>
+      <c r="J91" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K91" s="2" t="n"/>
       <c r="L91" s="2" t="inlineStr">
         <is>
@@ -7764,7 +7786,9 @@
       <c r="I92" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J92" s="2" t="n"/>
+      <c r="J92" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K92" s="2" t="n"/>
       <c r="L92" s="2" t="inlineStr">
         <is>
@@ -7815,7 +7839,9 @@
       <c r="I93" s="2" t="n">
         <v>13000</v>
       </c>
-      <c r="J93" s="2" t="n"/>
+      <c r="J93" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K93" s="2" t="n"/>
       <c r="L93" s="2" t="inlineStr">
         <is>
@@ -7866,7 +7892,9 @@
       <c r="I94" s="2" t="n">
         <v>13000</v>
       </c>
-      <c r="J94" s="2" t="n"/>
+      <c r="J94" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K94" s="2" t="n"/>
       <c r="L94" s="2" t="inlineStr">
         <is>
@@ -7917,7 +7945,9 @@
       <c r="I95" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J95" s="2" t="n"/>
+      <c r="J95" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K95" s="2" t="n"/>
       <c r="L95" s="2" t="inlineStr">
         <is>
@@ -7968,7 +7998,9 @@
       <c r="I96" s="2" t="n">
         <v>13500</v>
       </c>
-      <c r="J96" s="2" t="n"/>
+      <c r="J96" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K96" s="2" t="n"/>
       <c r="L96" s="2" t="inlineStr">
         <is>
@@ -8015,7 +8047,9 @@
       <c r="I97" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J97" s="2" t="n"/>
+      <c r="J97" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K97" s="2" t="n"/>
       <c r="L97" s="2" t="inlineStr">
         <is>
@@ -8066,7 +8100,9 @@
       <c r="I98" s="2" t="n">
         <v>6500</v>
       </c>
-      <c r="J98" s="2" t="n"/>
+      <c r="J98" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K98" s="2" t="n"/>
       <c r="L98" s="2" t="inlineStr">
         <is>
@@ -8117,7 +8153,9 @@
       <c r="I99" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J99" s="2" t="n"/>
+      <c r="J99" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K99" s="2" t="n"/>
       <c r="L99" s="2" t="inlineStr">
         <is>
@@ -8168,7 +8206,9 @@
       <c r="I100" s="2" t="n">
         <v>4000</v>
       </c>
-      <c r="J100" s="2" t="n"/>
+      <c r="J100" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K100" s="2" t="n"/>
       <c r="L100" s="2" t="inlineStr">
         <is>
@@ -8219,7 +8259,9 @@
       <c r="I101" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J101" s="2" t="n"/>
+      <c r="J101" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K101" s="2" t="n"/>
       <c r="L101" s="2" t="inlineStr">
         <is>
@@ -8270,7 +8312,9 @@
       <c r="I102" s="2" t="n">
         <v>4500</v>
       </c>
-      <c r="J102" s="2" t="n"/>
+      <c r="J102" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K102" s="2" t="n"/>
       <c r="L102" s="2" t="inlineStr">
         <is>
@@ -8321,7 +8365,9 @@
       <c r="I103" s="2" t="n">
         <v>2800</v>
       </c>
-      <c r="J103" s="2" t="n"/>
+      <c r="J103" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K103" s="2" t="n"/>
       <c r="L103" s="2" t="inlineStr">
         <is>
@@ -8372,7 +8418,9 @@
       <c r="I104" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J104" s="2" t="n"/>
+      <c r="J104" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K104" s="2" t="n"/>
       <c r="L104" s="2" t="inlineStr">
         <is>
@@ -8423,7 +8471,9 @@
       <c r="I105" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J105" s="2" t="n"/>
+      <c r="J105" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K105" s="2" t="n"/>
       <c r="L105" s="2" t="inlineStr">
         <is>
@@ -8474,7 +8524,9 @@
       <c r="I106" s="2" t="n">
         <v>1700</v>
       </c>
-      <c r="J106" s="2" t="n"/>
+      <c r="J106" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K106" s="2" t="n"/>
       <c r="L106" s="2" t="inlineStr">
         <is>
@@ -8525,7 +8577,9 @@
       <c r="I107" s="2" t="n">
         <v>1700</v>
       </c>
-      <c r="J107" s="2" t="n"/>
+      <c r="J107" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K107" s="2" t="n"/>
       <c r="L107" s="2" t="inlineStr">
         <is>
@@ -8576,7 +8630,9 @@
       <c r="I108" s="2" t="n">
         <v>1700</v>
       </c>
-      <c r="J108" s="2" t="n"/>
+      <c r="J108" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K108" s="2" t="n"/>
       <c r="L108" s="2" t="inlineStr">
         <is>
@@ -8627,7 +8683,9 @@
       <c r="I109" s="2" t="n">
         <v>1700</v>
       </c>
-      <c r="J109" s="2" t="n"/>
+      <c r="J109" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K109" s="2" t="n"/>
       <c r="L109" s="2" t="inlineStr">
         <is>
@@ -8678,7 +8736,9 @@
       <c r="I110" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="J110" s="2" t="n"/>
+      <c r="J110" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K110" s="2" t="n"/>
       <c r="L110" s="2" t="inlineStr">
         <is>
@@ -8729,7 +8789,9 @@
       <c r="I111" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="J111" s="2" t="n"/>
+      <c r="J111" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K111" s="2" t="n"/>
       <c r="L111" s="2" t="inlineStr">
         <is>
@@ -8780,7 +8842,9 @@
       <c r="I112" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J112" s="2" t="n"/>
+      <c r="J112" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K112" s="2" t="n"/>
       <c r="L112" s="2" t="inlineStr">
         <is>
@@ -8831,7 +8895,9 @@
       <c r="I113" s="2" t="n">
         <v>7000</v>
       </c>
-      <c r="J113" s="2" t="n"/>
+      <c r="J113" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K113" s="2" t="n"/>
       <c r="L113" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rebuild master_control.xlsx with pulled Ozon stock
data/ozon_catalog.xlsx now has real stock (FBO+FBS present) for all 68
existing products, pulled via pull-ozon-stock; master_control.xlsx's
"Остаток, шт." column now reflects it. Draft quantities (50, mechatronic
DQ250-with-board = 3) already applied last commit.
</commit_message>
<xml_diff>
--- a/data/master_control.xlsx
+++ b/data/master_control.xlsx
@@ -3157,7 +3157,9 @@
       <c r="I2" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="J2" s="2" t="n">
+        <v>90</v>
+      </c>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -3204,7 +3206,9 @@
       <c r="I3" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="J3" s="2" t="n"/>
+      <c r="J3" s="2" t="n">
+        <v>100</v>
+      </c>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -3255,7 +3259,9 @@
       <c r="I4" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J4" s="2" t="n"/>
+      <c r="J4" s="2" t="n">
+        <v>95</v>
+      </c>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
@@ -3359,7 +3365,9 @@
       <c r="I6" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="J6" s="2" t="n"/>
+      <c r="J6" s="2" t="n">
+        <v>87</v>
+      </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
@@ -3410,7 +3418,9 @@
       <c r="I7" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J7" s="2" t="n"/>
+      <c r="J7" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
@@ -3461,7 +3471,9 @@
       <c r="I8" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J8" s="2" t="n"/>
+      <c r="J8" s="2" t="n">
+        <v>11</v>
+      </c>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
@@ -3566,7 +3578,9 @@
       <c r="I10" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J10" s="2" t="n"/>
+      <c r="J10" s="2" t="n">
+        <v>19</v>
+      </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
@@ -3617,7 +3631,9 @@
       <c r="I11" s="2" t="n">
         <v>4500</v>
       </c>
-      <c r="J11" s="2" t="n"/>
+      <c r="J11" s="2" t="n">
+        <v>49</v>
+      </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
@@ -3668,7 +3684,9 @@
       <c r="I12" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J12" s="2" t="n"/>
+      <c r="J12" s="2" t="n">
+        <v>83</v>
+      </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
@@ -3719,7 +3737,9 @@
       <c r="I13" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="J13" s="2" t="n"/>
+      <c r="J13" s="2" t="n">
+        <v>87</v>
+      </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
@@ -3770,7 +3790,9 @@
       <c r="I14" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="J14" s="2" t="n"/>
+      <c r="J14" s="2" t="n">
+        <v>51</v>
+      </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
@@ -3825,7 +3847,9 @@
       <c r="I15" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="J15" s="2" t="n"/>
+      <c r="J15" s="2" t="n">
+        <v>35</v>
+      </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
@@ -3876,7 +3900,9 @@
       <c r="I16" s="2" t="n">
         <v>15000</v>
       </c>
-      <c r="J16" s="2" t="n"/>
+      <c r="J16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
@@ -3927,7 +3953,9 @@
       <c r="I17" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J17" s="2" t="n"/>
+      <c r="J17" s="2" t="n">
+        <v>28</v>
+      </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
@@ -3978,7 +4006,9 @@
       <c r="I18" s="2" t="n">
         <v>80000</v>
       </c>
-      <c r="J18" s="2" t="n"/>
+      <c r="J18" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
@@ -4029,7 +4059,9 @@
       <c r="I19" s="2" t="n">
         <v>4500</v>
       </c>
-      <c r="J19" s="2" t="n"/>
+      <c r="J19" s="2" t="n">
+        <v>51</v>
+      </c>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -4076,7 +4108,9 @@
       <c r="I20" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J20" s="2" t="n"/>
+      <c r="J20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
@@ -4127,7 +4161,9 @@
       <c r="I21" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="J21" s="2" t="n"/>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
@@ -4178,7 +4214,9 @@
       <c r="I22" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="J22" s="2" t="n"/>
+      <c r="J22" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
@@ -4396,7 +4434,9 @@
       <c r="I26" s="2" t="n">
         <v>18000</v>
       </c>
-      <c r="J26" s="2" t="n"/>
+      <c r="J26" s="2" t="n">
+        <v>25</v>
+      </c>
       <c r="K26" s="2" t="n"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
@@ -4447,7 +4487,9 @@
       <c r="I27" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="J27" s="2" t="n"/>
+      <c r="J27" s="2" t="n">
+        <v>74</v>
+      </c>
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="inlineStr">
         <is>
@@ -4498,7 +4540,9 @@
       <c r="I28" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J28" s="2" t="n"/>
+      <c r="J28" s="2" t="n">
+        <v>93</v>
+      </c>
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
@@ -4545,7 +4589,9 @@
       <c r="I29" s="2" t="n">
         <v>90000</v>
       </c>
-      <c r="J29" s="2" t="n"/>
+      <c r="J29" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -4658,7 +4704,9 @@
       <c r="I31" s="2" t="n">
         <v>150000</v>
       </c>
-      <c r="J31" s="2" t="n"/>
+      <c r="J31" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -4713,7 +4761,9 @@
       <c r="I32" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="J32" s="2" t="n"/>
+      <c r="J32" s="2" t="n">
+        <v>69</v>
+      </c>
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
@@ -4823,7 +4873,9 @@
       <c r="I34" s="2" t="n">
         <v>8000</v>
       </c>
-      <c r="J34" s="2" t="n"/>
+      <c r="J34" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
@@ -4878,7 +4930,9 @@
       <c r="I35" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J35" s="2" t="n"/>
+      <c r="J35" s="2" t="n">
+        <v>43</v>
+      </c>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
@@ -4929,7 +4983,9 @@
       <c r="I36" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="J36" s="2" t="n"/>
+      <c r="J36" s="2" t="n">
+        <v>93</v>
+      </c>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
@@ -4980,7 +5036,9 @@
       <c r="I37" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="J37" s="2" t="n"/>
+      <c r="J37" s="2" t="n">
+        <v>88</v>
+      </c>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
@@ -5035,7 +5093,9 @@
       <c r="I38" s="2" t="n">
         <v>2300</v>
       </c>
-      <c r="J38" s="2" t="n"/>
+      <c r="J38" s="2" t="n">
+        <v>86</v>
+      </c>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
@@ -5086,7 +5146,9 @@
       <c r="I39" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J39" s="2" t="n"/>
+      <c r="J39" s="2" t="n">
+        <v>74</v>
+      </c>
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
@@ -5137,7 +5199,9 @@
       <c r="I40" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J40" s="2" t="n"/>
+      <c r="J40" s="2" t="n">
+        <v>25</v>
+      </c>
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
@@ -5188,7 +5252,9 @@
       <c r="I41" s="2" t="n">
         <v>1800</v>
       </c>
-      <c r="J41" s="2" t="n"/>
+      <c r="J41" s="2" t="n">
+        <v>53</v>
+      </c>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
@@ -5239,7 +5305,9 @@
       <c r="I42" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J42" s="2" t="n"/>
+      <c r="J42" s="2" t="n">
+        <v>36</v>
+      </c>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
@@ -5290,7 +5358,9 @@
       <c r="I43" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J43" s="2" t="n"/>
+      <c r="J43" s="2" t="n">
+        <v>82</v>
+      </c>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
@@ -5337,7 +5407,9 @@
       <c r="I44" s="2" t="n">
         <v>90000</v>
       </c>
-      <c r="J44" s="2" t="n"/>
+      <c r="J44" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
@@ -5392,7 +5464,9 @@
       <c r="I45" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J45" s="2" t="n"/>
+      <c r="J45" s="2" t="n">
+        <v>47</v>
+      </c>
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
@@ -5518,7 +5592,9 @@
       <c r="I47" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="J47" s="2" t="n"/>
+      <c r="J47" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
@@ -5569,7 +5645,9 @@
       <c r="I48" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J48" s="2" t="n"/>
+      <c r="J48" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
@@ -5620,7 +5698,9 @@
       <c r="I49" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="J49" s="2" t="n"/>
+      <c r="J49" s="2" t="n">
+        <v>21</v>
+      </c>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
@@ -5671,7 +5751,9 @@
       <c r="I50" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="J50" s="2" t="n"/>
+      <c r="J50" s="2" t="n">
+        <v>49</v>
+      </c>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
@@ -5722,7 +5804,9 @@
       <c r="I51" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="J51" s="2" t="n"/>
+      <c r="J51" s="2" t="n">
+        <v>40</v>
+      </c>
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
@@ -5830,7 +5914,9 @@
       <c r="I53" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="J53" s="2" t="n"/>
+      <c r="J53" s="2" t="n">
+        <v>29</v>
+      </c>
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
@@ -5934,7 +6020,9 @@
       <c r="I55" s="2" t="n">
         <v>4000</v>
       </c>
-      <c r="J55" s="2" t="n"/>
+      <c r="J55" s="2" t="n">
+        <v>12</v>
+      </c>
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="inlineStr">
         <is>
@@ -5981,7 +6069,9 @@
       <c r="I56" s="2" t="n">
         <v>15000</v>
       </c>
-      <c r="J56" s="2" t="n"/>
+      <c r="J56" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
@@ -6028,7 +6118,9 @@
       <c r="I57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J57" s="2" t="n"/>
+      <c r="J57" s="2" t="n">
+        <v>49</v>
+      </c>
       <c r="K57" s="2" t="n"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
@@ -6079,7 +6171,9 @@
       <c r="I58" s="2" t="n">
         <v>25000</v>
       </c>
-      <c r="J58" s="2" t="n"/>
+      <c r="J58" s="2" t="n">
+        <v>80</v>
+      </c>
       <c r="K58" s="2" t="n"/>
       <c r="L58" s="2" t="inlineStr">
         <is>
@@ -6130,7 +6224,9 @@
       <c r="I59" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J59" s="2" t="n"/>
+      <c r="J59" s="2" t="n">
+        <v>49</v>
+      </c>
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="inlineStr">
         <is>
@@ -6181,7 +6277,9 @@
       <c r="I60" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="J60" s="2" t="n"/>
+      <c r="J60" s="2" t="n">
+        <v>53</v>
+      </c>
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="inlineStr">
         <is>
@@ -6232,7 +6330,9 @@
       <c r="I61" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J61" s="2" t="n"/>
+      <c r="J61" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K61" s="2" t="n"/>
       <c r="L61" s="2" t="inlineStr">
         <is>
@@ -6283,7 +6383,9 @@
       <c r="I62" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J62" s="2" t="n"/>
+      <c r="J62" s="2" t="n">
+        <v>32</v>
+      </c>
       <c r="K62" s="2" t="n"/>
       <c r="L62" s="2" t="inlineStr">
         <is>
@@ -6334,7 +6436,9 @@
       <c r="I63" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J63" s="2" t="n"/>
+      <c r="J63" s="2" t="n">
+        <v>36</v>
+      </c>
       <c r="K63" s="2" t="n"/>
       <c r="L63" s="2" t="inlineStr">
         <is>
@@ -6385,7 +6489,9 @@
       <c r="I64" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="J64" s="2" t="n"/>
+      <c r="J64" s="2" t="n">
+        <v>28</v>
+      </c>
       <c r="K64" s="2" t="n"/>
       <c r="L64" s="2" t="inlineStr">
         <is>
@@ -6436,7 +6542,9 @@
       <c r="I65" s="2" t="n">
         <v>80000</v>
       </c>
-      <c r="J65" s="2" t="n"/>
+      <c r="J65" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K65" s="2" t="n"/>
       <c r="L65" s="2" t="inlineStr">
         <is>
@@ -6553,7 +6661,9 @@
       <c r="I67" s="2" t="n">
         <v>80000</v>
       </c>
-      <c r="J67" s="2" t="n"/>
+      <c r="J67" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K67" s="2" t="n"/>
       <c r="L67" s="2" t="inlineStr">
         <is>
@@ -6608,7 +6718,9 @@
       <c r="I68" s="2" t="n">
         <v>80000</v>
       </c>
-      <c r="J68" s="2" t="n"/>
+      <c r="J68" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="K68" s="2" t="n"/>
       <c r="L68" s="2" t="inlineStr">
         <is>
@@ -6659,7 +6771,9 @@
       <c r="I69" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="J69" s="2" t="n"/>
+      <c r="J69" s="2" t="n">
+        <v>37</v>
+      </c>
       <c r="K69" s="2" t="n"/>
       <c r="L69" s="2" t="inlineStr">
         <is>
@@ -6841,7 +6955,9 @@
       <c r="I73" s="2" t="n">
         <v>8000</v>
       </c>
-      <c r="J73" s="2" t="n"/>
+      <c r="J73" s="2" t="n">
+        <v>50</v>
+      </c>
       <c r="K73" s="2" t="n"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
@@ -6888,7 +7004,9 @@
       <c r="I74" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J74" s="2" t="n"/>
+      <c r="J74" s="2" t="n">
+        <v>44</v>
+      </c>
       <c r="K74" s="2" t="n"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
@@ -6939,7 +7057,9 @@
       <c r="I75" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="J75" s="2" t="n"/>
+      <c r="J75" s="2" t="n">
+        <v>77</v>
+      </c>
       <c r="K75" s="2" t="n"/>
       <c r="L75" s="2" t="inlineStr">
         <is>
@@ -6986,7 +7106,9 @@
       <c r="I76" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J76" s="2" t="n"/>
+      <c r="J76" s="2" t="n">
+        <v>30</v>
+      </c>
       <c r="K76" s="2" t="n"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
@@ -7033,7 +7155,9 @@
       <c r="I77" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="J77" s="2" t="n"/>
+      <c r="J77" s="2" t="n">
+        <v>19</v>
+      </c>
       <c r="K77" s="2" t="n"/>
       <c r="L77" s="2" t="inlineStr">
         <is>
@@ -7084,7 +7208,9 @@
       <c r="I78" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="J78" s="2" t="n"/>
+      <c r="J78" s="2" t="n">
+        <v>30</v>
+      </c>
       <c r="K78" s="2" t="n"/>
       <c r="L78" s="2" t="inlineStr">
         <is>
@@ -7131,7 +7257,9 @@
       <c r="I79" s="2" t="n">
         <v>3500</v>
       </c>
-      <c r="J79" s="2" t="n"/>
+      <c r="J79" s="2" t="n">
+        <v>16</v>
+      </c>
       <c r="K79" s="2" t="n"/>
       <c r="L79" s="2" t="inlineStr">
         <is>
@@ -7178,7 +7306,9 @@
       <c r="I80" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J80" s="2" t="n"/>
+      <c r="J80" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K80" s="2" t="n"/>
       <c r="L80" s="2" t="inlineStr">
         <is>
@@ -7270,7 +7400,9 @@
       <c r="I82" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J82" s="2" t="n"/>
+      <c r="J82" s="2" t="n">
+        <v>93</v>
+      </c>
       <c r="K82" s="2" t="n"/>
       <c r="L82" s="2" t="inlineStr">
         <is>
@@ -7427,7 +7559,9 @@
       <c r="I85" s="2" t="n">
         <v>15000</v>
       </c>
-      <c r="J85" s="2" t="n"/>
+      <c r="J85" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K85" s="2" t="n"/>
       <c r="L85" s="2" t="inlineStr">
         <is>
@@ -7580,7 +7714,9 @@
       <c r="I88" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="J88" s="2" t="n"/>
+      <c r="J88" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="K88" s="2" t="n"/>
       <c r="L88" s="2" t="inlineStr">
         <is>

</xml_diff>